<commit_message>
crypto-cex: spell out concrete UI steps for FE/UI cases in TestCases.xlsx (screen, URL, navigation, on-screen check)
</commit_message>
<xml_diff>
--- a/testcases/TestCases.xlsx
+++ b/testcases/TestCases.xlsx
@@ -3099,8 +3099,9 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Then the assets on screen include BTC, ETH, SOL, USD
-And every asset row on screen shows a symbol and a USD price</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. On screen, verify: the assets on screen include BTC, ETH, SOL, USD.
+3. On screen, verify: every asset row on screen shows a symbol and a USD price.</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -3151,7 +3152,8 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Then the DOGE row on screen is marked delisted</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. On screen, verify: the DOGE row on screen is marked delisted.</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
@@ -3201,7 +3203,8 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Then the number of assets on screen equals the API asset count</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. On screen, verify: the number of assets on screen equals the API asset count.</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -3251,9 +3254,10 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 1.0 BTC
-When the wallet page for "alice" is opened
-Then the BTC balance on screen is 1.0</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 1.0 BTC.
+3. Open the app 'Wallet' screen in the browser (URL /wallet/&lt;account&gt;) — open the account's wallet page.
+4. On screen, verify: the BTC balance on screen is 1.0.</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
@@ -3303,9 +3307,10 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 2.0 ETH
-When the wallet page for "alice" is opened
-Then every balance on screen matches the API balance for "alice"</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 2.0 ETH.
+3. Open the app 'Wallet' screen in the browser (URL /wallet/&lt;account&gt;) — open the account's wallet page.
+4. On screen, verify: every balance on screen matches the API balance for "alice".</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
@@ -3355,10 +3360,11 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 1.0 BTC
-And "alice" bridge-withdraws 0.2 BTC to chain "ethereum"
-When the op page for that bridge op is opened
-Then the op status on screen is "locked"</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 1.0 BTC.
+3. Set up (before checking the screen): "alice" bridge-withdraws 0.2 BTC to chain "ethereum".
+4. Open the app 'Bridge op' screen in the browser (URL /op/&lt;opId&gt;) — click the bridge op just created.
+5. On screen, verify: the op status on screen is "locked".</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
@@ -3408,11 +3414,12 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 1.0 BTC
-And a fresh account "bob"
-When the transfer form is submitted moving 0.4 BTC from "alice" to "bob"
-Then the form result status is 201
-And the API balance for "bob" in BTC is 0.4 BTC</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 1.0 BTC.
+3. Set up (before checking the screen): a fresh account "bob".
+4. Open the app 'Transfer panel' screen in the browser (URL / (Transfer)) — enter recipient and 0.4 BTC, click Send.
+5. On screen, verify: the form result status is 201.
+6. On screen, verify: the API balance for "bob" in BTC is 0.4 BTC.</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
@@ -3463,10 +3470,11 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 1.0 BTC
-When the swap form is submitted converting 0.5 BTC to USD for "alice"
-Then the form result status is 201
-And the API balance for "alice" in USD is above zero</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 1.0 BTC.
+3. Open the app 'Swap panel' screen in the browser (URL / (Swap)) — on the Swap panel, enter 0.5 BTC, choose USD, click Swap.
+4. On screen, verify: the form result status is 201.
+5. On screen, verify: the API balance for "alice" in USD is above zero.</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
@@ -3517,10 +3525,11 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 1.0 BTC
-When the bridge form is submitted withdrawing 0.3 BTC to chain "ethereum" for "alice"
-Then the form result status is 201
-And the form result code is "ok"</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 1.0 BTC.
+3. Open the app 'Bridge panel' screen in the browser (URL / (Bridge)) — choose chain "ethereum", enter 0.3 BTC, click Withdraw.
+4. On screen, verify: the form result status is 201.
+5. On screen, verify: the form result code is "ok".</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
@@ -3571,11 +3580,12 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>Given a fresh account "alice" funded with 0.1 BTC
-And a fresh account "bob"
-When the transfer form is submitted moving 9.0 BTC from "alice" to "bob"
-Then the form result status is 409
-And the form result code is "insufficient_funds"</t>
+          <t>1. Open the app 'Home / wallet' screen in the browser (URL /) — the app landing page.
+2. Set up (before checking the screen): a fresh account "alice" funded with 0.1 BTC.
+3. Set up (before checking the screen): a fresh account "bob".
+4. Open the app 'Transfer panel' screen in the browser (URL / (Transfer)) — enter recipient and 9.0 BTC, click Send.
+5. On screen, verify: the form result status is 409.
+6. On screen, verify: the form result code is "insufficient_funds".</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">

</xml_diff>